<commit_message>
add reference to the specific profile in imaging-related profiles cd28bfe1f5972af554772f9637092c4fe6596e36
</commit_message>
<xml_diff>
--- a/specific-profile-img/ig/StructureDefinition-fr-diagnostic-report-imaging-document.xlsx
+++ b/specific-profile-img/ig/StructureDefinition-fr-diagnostic-report-imaging-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-31T07:56:22+00:00</t>
+    <t>2026-07-31T09:38:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -609,7 +609,7 @@
     <t>serviceRequestAccessionNumber</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-service-request-document|0.1.0)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-service-request-imaging-document|0.1.0)
 </t>
   </si>
   <si>

</xml_diff>